<commit_message>
Rename energy into contraction power
</commit_message>
<xml_diff>
--- a/local/Datasheet_template_example.xlsx
+++ b/local/Datasheet_template_example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donatella.cea/Documents/Contraction analysis of neuromuscular organoids/NMOs-Contraction/local/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donatella.cea/Vouchers/Contraction analysis of neuromuscular organoids/NMOs-Contraction/local/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F260704-663F-1544-AADC-B64EBEACBFD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3098D2AF-2E81-CB4F-BBD9-F4BF8D350156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34100" yWindow="280" windowWidth="28800" windowHeight="16520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,9 +73,6 @@
     <t>Threshold organoid border</t>
   </si>
   <si>
-    <t>Energy</t>
-  </si>
-  <si>
     <t>Mean</t>
   </si>
   <si>
@@ -239,6 +236,9 @@
   </si>
   <si>
     <t>Total Area [mm^2]</t>
+  </si>
+  <si>
+    <t>Contraction power</t>
   </si>
 </sst>
 </file>
@@ -655,60 +655,60 @@
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>27</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>28</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2">
+        <v>65</v>
+      </c>
+      <c r="G2" t="s">
         <v>29</v>
       </c>
-      <c r="F2">
-        <v>65</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="K2" t="s">
         <v>30</v>
-      </c>
-      <c r="K2" t="s">
-        <v>31</v>
       </c>
       <c r="L2">
         <v>0.59</v>
@@ -752,28 +752,28 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>27</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>28</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3">
+        <v>65</v>
+      </c>
+      <c r="G3" t="s">
         <v>29</v>
       </c>
-      <c r="F3">
-        <v>65</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="K3" t="s">
         <v>30</v>
-      </c>
-      <c r="K3" t="s">
-        <v>31</v>
       </c>
       <c r="L3">
         <v>0.59</v>
@@ -817,28 +817,28 @@
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4">
+        <v>65</v>
+      </c>
+      <c r="G4" t="s">
         <v>29</v>
       </c>
-      <c r="F4">
-        <v>65</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="K4" t="s">
         <v>30</v>
-      </c>
-      <c r="K4" t="s">
-        <v>31</v>
       </c>
       <c r="L4">
         <v>0.59</v>
@@ -882,28 +882,28 @@
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>27</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>28</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5">
+        <v>65</v>
+      </c>
+      <c r="G5" t="s">
         <v>29</v>
       </c>
-      <c r="F5">
-        <v>65</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="K5" t="s">
         <v>30</v>
-      </c>
-      <c r="K5" t="s">
-        <v>31</v>
       </c>
       <c r="L5">
         <v>0.59</v>
@@ -947,28 +947,28 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>27</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>28</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6">
+        <v>65</v>
+      </c>
+      <c r="G6" t="s">
         <v>29</v>
       </c>
-      <c r="F6">
-        <v>65</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="K6" t="s">
         <v>30</v>
-      </c>
-      <c r="K6" t="s">
-        <v>31</v>
       </c>
       <c r="L6">
         <v>0.59</v>
@@ -1012,28 +1012,28 @@
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>28</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7">
+        <v>65</v>
+      </c>
+      <c r="G7" t="s">
         <v>29</v>
       </c>
-      <c r="F7">
-        <v>65</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="K7" t="s">
         <v>30</v>
-      </c>
-      <c r="K7" t="s">
-        <v>31</v>
       </c>
       <c r="L7">
         <v>0.59</v>
@@ -1077,28 +1077,28 @@
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
         <v>26</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>27</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>28</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8">
+        <v>65</v>
+      </c>
+      <c r="G8" t="s">
         <v>29</v>
       </c>
-      <c r="F8">
-        <v>65</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="K8" t="s">
         <v>30</v>
-      </c>
-      <c r="K8" t="s">
-        <v>31</v>
       </c>
       <c r="L8">
         <v>0.59</v>
@@ -1142,28 +1142,28 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>27</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>28</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9">
+        <v>65</v>
+      </c>
+      <c r="G9" t="s">
         <v>29</v>
       </c>
-      <c r="F9">
-        <v>65</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="K9" t="s">
         <v>30</v>
-      </c>
-      <c r="K9" t="s">
-        <v>31</v>
       </c>
       <c r="L9">
         <v>0.59</v>
@@ -1207,28 +1207,28 @@
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10">
+        <v>65</v>
+      </c>
+      <c r="G10" t="s">
+        <v>29</v>
+      </c>
+      <c r="K10" t="s">
         <v>39</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10">
-        <v>65</v>
-      </c>
-      <c r="G10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K10" t="s">
-        <v>40</v>
       </c>
       <c r="L10">
         <v>0.39</v>
@@ -1272,28 +1272,28 @@
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
         <v>26</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>28</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11">
+        <v>65</v>
+      </c>
+      <c r="G11" t="s">
         <v>29</v>
       </c>
-      <c r="F11">
-        <v>65</v>
-      </c>
-      <c r="G11" t="s">
-        <v>30</v>
-      </c>
       <c r="K11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L11">
         <v>0.39</v>
@@ -1337,28 +1337,28 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>27</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>28</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12">
+        <v>65</v>
+      </c>
+      <c r="G12" t="s">
         <v>29</v>
       </c>
-      <c r="F12">
-        <v>65</v>
-      </c>
-      <c r="G12" t="s">
-        <v>30</v>
-      </c>
       <c r="K12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L12">
         <v>0.39</v>
@@ -1402,28 +1402,28 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13">
+        <v>65</v>
+      </c>
+      <c r="G13" t="s">
+        <v>29</v>
+      </c>
+      <c r="K13" t="s">
         <v>43</v>
-      </c>
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" t="s">
-        <v>28</v>
-      </c>
-      <c r="E13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F13">
-        <v>65</v>
-      </c>
-      <c r="G13" t="s">
-        <v>30</v>
-      </c>
-      <c r="K13" t="s">
-        <v>44</v>
       </c>
       <c r="L13">
         <v>0.56999999999999995</v>
@@ -1467,28 +1467,28 @@
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
         <v>26</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>27</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>28</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14">
+        <v>65</v>
+      </c>
+      <c r="G14" t="s">
         <v>29</v>
       </c>
-      <c r="F14">
-        <v>65</v>
-      </c>
-      <c r="G14" t="s">
-        <v>30</v>
-      </c>
       <c r="K14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L14">
         <v>0.56999999999999995</v>
@@ -1532,28 +1532,28 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" t="s">
         <v>26</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>27</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>28</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15">
+        <v>65</v>
+      </c>
+      <c r="G15" t="s">
         <v>29</v>
       </c>
-      <c r="F15">
-        <v>65</v>
-      </c>
-      <c r="G15" t="s">
-        <v>30</v>
-      </c>
       <c r="K15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L15">
         <v>0.56999999999999995</v>
@@ -1597,28 +1597,28 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" t="s">
         <v>26</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>27</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>28</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16">
+        <v>65</v>
+      </c>
+      <c r="G16" t="s">
         <v>29</v>
       </c>
-      <c r="F16">
-        <v>65</v>
-      </c>
-      <c r="G16" t="s">
-        <v>30</v>
-      </c>
       <c r="K16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L16">
         <v>0.56999999999999995</v>
@@ -1662,28 +1662,28 @@
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" t="s">
         <v>26</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>27</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>28</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17">
+        <v>65</v>
+      </c>
+      <c r="G17" t="s">
         <v>29</v>
       </c>
-      <c r="F17">
-        <v>65</v>
-      </c>
-      <c r="G17" t="s">
-        <v>30</v>
-      </c>
       <c r="K17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L17">
         <v>0.56999999999999995</v>
@@ -1727,28 +1727,28 @@
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" t="s">
         <v>26</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>27</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>28</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18">
+        <v>65</v>
+      </c>
+      <c r="G18" t="s">
         <v>29</v>
       </c>
-      <c r="F18">
-        <v>65</v>
-      </c>
-      <c r="G18" t="s">
-        <v>30</v>
-      </c>
       <c r="K18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L18">
         <v>0.56999999999999995</v>
@@ -1792,28 +1792,28 @@
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
         <v>26</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>27</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>28</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19">
+        <v>65</v>
+      </c>
+      <c r="G19" t="s">
         <v>29</v>
       </c>
-      <c r="F19">
-        <v>65</v>
-      </c>
-      <c r="G19" t="s">
-        <v>30</v>
-      </c>
       <c r="K19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L19">
         <v>0.56999999999999995</v>
@@ -1857,28 +1857,28 @@
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20">
+        <v>65</v>
+      </c>
+      <c r="G20" t="s">
+        <v>29</v>
+      </c>
+      <c r="K20" t="s">
         <v>51</v>
-      </c>
-      <c r="B20" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" t="s">
-        <v>29</v>
-      </c>
-      <c r="F20">
-        <v>65</v>
-      </c>
-      <c r="G20" t="s">
-        <v>30</v>
-      </c>
-      <c r="K20" t="s">
-        <v>52</v>
       </c>
       <c r="L20">
         <v>0.55000000000000004</v>
@@ -1922,28 +1922,28 @@
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" t="s">
         <v>26</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>27</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>28</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21">
+        <v>65</v>
+      </c>
+      <c r="G21" t="s">
         <v>29</v>
       </c>
-      <c r="F21">
-        <v>65</v>
-      </c>
-      <c r="G21" t="s">
-        <v>30</v>
-      </c>
       <c r="K21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L21">
         <v>0.55000000000000004</v>
@@ -1987,28 +1987,28 @@
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" t="s">
         <v>26</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>27</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>28</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22">
+        <v>65</v>
+      </c>
+      <c r="G22" t="s">
         <v>29</v>
       </c>
-      <c r="F22">
-        <v>65</v>
-      </c>
-      <c r="G22" t="s">
-        <v>30</v>
-      </c>
       <c r="K22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L22">
         <v>0.55000000000000004</v>
@@ -2052,28 +2052,28 @@
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" t="s">
         <v>26</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>27</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>28</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23">
+        <v>65</v>
+      </c>
+      <c r="G23" t="s">
         <v>29</v>
       </c>
-      <c r="F23">
-        <v>65</v>
-      </c>
-      <c r="G23" t="s">
-        <v>30</v>
-      </c>
       <c r="K23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L23">
         <v>0.55000000000000004</v>
@@ -2117,28 +2117,28 @@
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" t="s">
         <v>26</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>27</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>28</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24">
+        <v>65</v>
+      </c>
+      <c r="G24" t="s">
         <v>29</v>
       </c>
-      <c r="F24">
-        <v>65</v>
-      </c>
-      <c r="G24" t="s">
-        <v>30</v>
-      </c>
       <c r="K24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L24">
         <v>0.55000000000000004</v>
@@ -2182,28 +2182,28 @@
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" t="s">
         <v>26</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>27</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>28</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25">
+        <v>65</v>
+      </c>
+      <c r="G25" t="s">
         <v>29</v>
       </c>
-      <c r="F25">
-        <v>65</v>
-      </c>
-      <c r="G25" t="s">
-        <v>30</v>
-      </c>
       <c r="K25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L25">
         <v>0.55000000000000004</v>
@@ -2247,28 +2247,28 @@
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
         <v>26</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>27</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>28</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26">
+        <v>65</v>
+      </c>
+      <c r="G26" t="s">
         <v>29</v>
       </c>
-      <c r="F26">
-        <v>65</v>
-      </c>
-      <c r="G26" t="s">
-        <v>30</v>
-      </c>
       <c r="K26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L26">
         <v>0.55000000000000004</v>
@@ -2312,28 +2312,28 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
         <v>26</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>27</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>28</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27">
+        <v>65</v>
+      </c>
+      <c r="G27" t="s">
         <v>29</v>
       </c>
-      <c r="F27">
-        <v>65</v>
-      </c>
-      <c r="G27" t="s">
-        <v>30</v>
-      </c>
       <c r="K27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L27">
         <v>0.55000000000000004</v>
@@ -2377,28 +2377,28 @@
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" t="s">
         <v>60</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>61</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
+        <v>61</v>
+      </c>
+      <c r="E28" t="s">
         <v>62</v>
-      </c>
-      <c r="D28" t="s">
-        <v>62</v>
-      </c>
-      <c r="E28" t="s">
-        <v>63</v>
       </c>
       <c r="F28">
         <v>58</v>
       </c>
       <c r="G28" t="s">
+        <v>63</v>
+      </c>
+      <c r="K28" t="s">
         <v>64</v>
-      </c>
-      <c r="K28" t="s">
-        <v>65</v>
       </c>
       <c r="L28">
         <v>0.44</v>
@@ -2424,28 +2424,28 @@
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" t="s">
+        <v>61</v>
+      </c>
+      <c r="E29" t="s">
         <v>66</v>
-      </c>
-      <c r="B29" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" t="s">
-        <v>62</v>
-      </c>
-      <c r="D29" t="s">
-        <v>62</v>
-      </c>
-      <c r="E29" t="s">
-        <v>67</v>
       </c>
       <c r="F29">
         <v>54</v>
       </c>
       <c r="G29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L29">
         <v>0.42</v>
@@ -2471,28 +2471,28 @@
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B30" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" t="s">
         <v>61</v>
       </c>
-      <c r="C30" t="s">
-        <v>62</v>
-      </c>
       <c r="D30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F30">
         <v>54</v>
       </c>
       <c r="G30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L30">
         <v>0.1</v>
@@ -2518,7 +2518,7 @@
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="T31">
         <v>0.28999999999999998</v>
@@ -2541,7 +2541,7 @@
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.2">
       <c r="K32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L32">
         <v>0.28999999999999998</v>
@@ -2564,7 +2564,7 @@
     </row>
     <row r="33" spans="11:26" x14ac:dyDescent="0.2">
       <c r="K33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L33">
         <v>0.28999999999999998</v>

</xml_diff>

<commit_message>
clean datasheet from wrong entries
</commit_message>
<xml_diff>
--- a/local/Datasheet_template_example.xlsx
+++ b/local/Datasheet_template_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donatella.cea/Vouchers/Contraction analysis of neuromuscular organoids/NMOs-Contraction/local/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3098D2AF-2E81-CB4F-BBD9-F4BF8D350156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6004785D-FF64-8D47-A19D-EB474C52705C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34100" yWindow="280" windowWidth="28800" windowHeight="16520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35260" yWindow="-320" windowWidth="28820" windowHeight="16540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="74">
   <si>
     <t>Video name</t>
   </si>
@@ -232,13 +232,16 @@
     <t>P1365_SMA_RISD_d54_O3</t>
   </si>
   <si>
-    <t>P1365_SMA_BRAN_d60_O4</t>
-  </si>
-  <si>
     <t>Total Area [mm^2]</t>
   </si>
   <si>
-    <t>Contraction power</t>
+    <t xml:space="preserve">Contraction power </t>
+  </si>
+  <si>
+    <t>Organoid</t>
+  </si>
+  <si>
+    <t>Position</t>
   </si>
 </sst>
 </file>
@@ -268,7 +271,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -291,13 +294,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -602,10 +619,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z33"/>
+  <dimension ref="A1:AB30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="31" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -655,13 +675,13 @@
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>17</v>
@@ -684,8 +704,14 @@
       <c r="Z1" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="AA1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -750,7 +776,7 @@
         <v>0.491052716</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -815,7 +841,7 @@
         <v>0.383282283</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -880,7 +906,7 @@
         <v>0.39053683700000003</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -945,7 +971,7 @@
         <v>0.49879090799999998</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1010,7 +1036,7 @@
         <v>0.45872964700000002</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -1075,7 +1101,7 @@
         <v>0.46751571800000002</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -1140,7 +1166,7 @@
         <v>0.45324842799999998</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1205,7 +1231,7 @@
         <v>0.44147992899999999</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1270,7 +1296,7 @@
         <v>0.56182492299999998</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1335,7 +1361,7 @@
         <v>0.46743511199999999</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -1400,7 +1426,7 @@
         <v>0.52571336499999999</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -1465,7 +1491,7 @@
         <v>0.46703208099999999</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -1530,7 +1556,7 @@
         <v>0.533290343</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>45</v>
       </c>
@@ -1595,7 +1621,7 @@
         <v>0.53740125699999997</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>46</v>
       </c>
@@ -1660,7 +1686,7 @@
         <v>0.58479767900000001</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -1725,7 +1751,7 @@
         <v>0.493954538</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1790,7 +1816,7 @@
         <v>0.50588425000000004</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>49</v>
       </c>
@@ -1855,7 +1881,7 @@
         <v>0.55078187999999995</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>50</v>
       </c>
@@ -1920,7 +1946,7 @@
         <v>0.44196356599999997</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -1985,7 +2011,7 @@
         <v>0.30678703899999998</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -2050,7 +2076,7 @@
         <v>0.30968886000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -2115,7 +2141,7 @@
         <v>0.52853457999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -2180,7 +2206,7 @@
         <v>0.78292761600000005</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>56</v>
       </c>
@@ -2245,7 +2271,7 @@
         <v>0.62348863499999996</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>57</v>
       </c>
@@ -2310,7 +2336,7 @@
         <v>0.52740609400000005</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>58</v>
       </c>
@@ -2375,7 +2401,7 @@
         <v>0.44575205499999998</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -2422,7 +2448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>65</v>
       </c>
@@ -2469,7 +2495,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>68</v>
       </c>
@@ -2514,75 +2540,6 @@
       </c>
       <c r="R30">
         <v>0.61</v>
-      </c>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="S31" t="s">
-        <v>70</v>
-      </c>
-      <c r="T31">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="U31">
-        <v>0.71</v>
-      </c>
-      <c r="V31">
-        <v>0.65981158088235292</v>
-      </c>
-      <c r="W31">
-        <v>0.23502604166666671</v>
-      </c>
-      <c r="X31">
-        <v>1</v>
-      </c>
-      <c r="Y31">
-        <v>56399</v>
-      </c>
-    </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="K32" t="s">
-        <v>70</v>
-      </c>
-      <c r="L32">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="M32">
-        <v>0.71</v>
-      </c>
-      <c r="N32">
-        <v>0.65981158088235292</v>
-      </c>
-      <c r="O32">
-        <v>0.23502604166666671</v>
-      </c>
-      <c r="P32">
-        <v>0</v>
-      </c>
-      <c r="Z32">
-        <v>2.09</v>
-      </c>
-    </row>
-    <row r="33" spans="11:26" x14ac:dyDescent="0.2">
-      <c r="K33" t="s">
-        <v>70</v>
-      </c>
-      <c r="L33">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="M33">
-        <v>0.71</v>
-      </c>
-      <c r="N33">
-        <v>0.65981158088235292</v>
-      </c>
-      <c r="O33">
-        <v>0.23502604166666671</v>
-      </c>
-      <c r="P33" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z33">
-        <v>2.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>